<commit_message>
Update Laydown module spreadsheet
</commit_message>
<xml_diff>
--- a/Laydown1_Module1.xlsx
+++ b/Laydown1_Module1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\material on laydown\outputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78B39164-BAA4-4B89-9C73-FBDAFA74BBCF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5E70BEB-946C-47BA-8367-EA47779BBD4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Zone5" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="944" uniqueCount="221">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="946" uniqueCount="222">
   <si>
     <t>Date</t>
   </si>
@@ -685,6 +685,9 @@
   </si>
   <si>
     <t>delivery on site</t>
+  </si>
+  <si>
+    <t>ME1-SB-188</t>
   </si>
 </sst>
 </file>
@@ -835,7 +838,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -881,6 +884,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1462,11 +1468,21 @@
       <c r="F15" s="14">
         <v>1</v>
       </c>
-      <c r="J15" s="5"/>
-      <c r="K15" s="8"/>
-      <c r="L15" s="8"/>
-      <c r="M15" s="5"/>
-      <c r="N15" s="8"/>
+      <c r="J15" s="16">
+        <v>46168</v>
+      </c>
+      <c r="K15" s="14">
+        <v>2605389</v>
+      </c>
+      <c r="L15" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="M15" s="13" t="s">
+        <v>221</v>
+      </c>
+      <c r="N15" s="15">
+        <v>1</v>
+      </c>
     </row>
     <row r="16" spans="2:14">
       <c r="B16" s="13" t="s">

</xml_diff>

<commit_message>
Update Laydown module 1 spreadsheet
</commit_message>
<xml_diff>
--- a/Laydown1_Module1.xlsx
+++ b/Laydown1_Module1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\material on laydown\outputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5E70BEB-946C-47BA-8367-EA47779BBD4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C21CAED5-25F2-416C-BC17-BFB9F233C498}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Zone5" sheetId="1" r:id="rId1"/>
@@ -2885,1492 +2885,1492 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="B3:K89"/>
+  <dimension ref="C3:L89"/>
   <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
-    <col min="1" max="1" width="2.69921875" customWidth="1"/>
-    <col min="2" max="2" width="11.8984375" customWidth="1"/>
-    <col min="3" max="3" width="11.19921875" customWidth="1"/>
-    <col min="4" max="4" width="15" customWidth="1"/>
-    <col min="5" max="5" width="16.19921875" customWidth="1"/>
-    <col min="6" max="6" width="6.8984375" customWidth="1"/>
-    <col min="8" max="9" width="2.69921875" customWidth="1"/>
-    <col min="10" max="10" width="11.8984375" customWidth="1"/>
-    <col min="11" max="11" width="13" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="15" customWidth="1"/>
-    <col min="13" max="13" width="16.19921875" customWidth="1"/>
-    <col min="14" max="14" width="6.8984375" customWidth="1"/>
-    <col min="15" max="15" width="2.69921875" customWidth="1"/>
+    <col min="2" max="2" width="2.69921875" customWidth="1"/>
+    <col min="3" max="3" width="11.8984375" customWidth="1"/>
+    <col min="4" max="4" width="11.19921875" customWidth="1"/>
+    <col min="5" max="5" width="17.69921875" customWidth="1"/>
+    <col min="6" max="6" width="16.19921875" customWidth="1"/>
+    <col min="7" max="7" width="6.8984375" customWidth="1"/>
+    <col min="9" max="10" width="2.69921875" customWidth="1"/>
+    <col min="11" max="11" width="11.8984375" customWidth="1"/>
+    <col min="12" max="12" width="13" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="15" customWidth="1"/>
+    <col min="14" max="14" width="16.19921875" customWidth="1"/>
+    <col min="15" max="15" width="6.8984375" customWidth="1"/>
+    <col min="16" max="16" width="2.69921875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:11">
-      <c r="B3" s="1" t="s">
+    <row r="3" spans="3:12">
+      <c r="C3" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>1</v>
-      </c>
       <c r="D3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="E3" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="F3" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="G3" s="3" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="2:11">
-      <c r="B4" s="13"/>
-      <c r="C4" s="14"/>
-      <c r="D4" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E4" s="13" t="s">
+    <row r="4" spans="3:12">
+      <c r="C4" s="13"/>
+      <c r="D4" s="14"/>
+      <c r="E4" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F4" s="13" t="s">
         <v>118</v>
       </c>
-      <c r="F4" s="14">
-        <v>1</v>
-      </c>
-      <c r="J4" s="12"/>
-      <c r="K4" s="8" t="s">
+      <c r="G4" s="14">
+        <v>1</v>
+      </c>
+      <c r="K4" s="12"/>
+      <c r="L4" s="8" t="s">
         <v>220</v>
       </c>
     </row>
-    <row r="5" spans="2:11">
-      <c r="B5" s="13" t="s">
+    <row r="5" spans="3:12">
+      <c r="C5" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="C5" s="14" t="s">
+      <c r="D5" s="14" t="s">
         <v>119</v>
       </c>
-      <c r="D5" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E5" s="13" t="s">
+      <c r="E5" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F5" s="13" t="s">
         <v>120</v>
       </c>
-      <c r="F5" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="2:11">
-      <c r="B6" s="13" t="s">
+      <c r="G5" s="15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="3:12">
+      <c r="C6" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="C6" s="14" t="s">
+      <c r="D6" s="14" t="s">
         <v>119</v>
       </c>
-      <c r="D6" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E6" s="13" t="s">
+      <c r="E6" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F6" s="13" t="s">
         <v>120</v>
       </c>
-      <c r="F6" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="2:11">
-      <c r="B7" s="13" t="s">
+      <c r="G6" s="15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="3:12">
+      <c r="C7" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="C7" s="14" t="s">
+      <c r="D7" s="14" t="s">
         <v>119</v>
       </c>
-      <c r="D7" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E7" s="13" t="s">
+      <c r="E7" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F7" s="13" t="s">
         <v>120</v>
       </c>
-      <c r="F7" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="2:11">
-      <c r="B8" s="13" t="s">
+      <c r="G7" s="15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="3:12">
+      <c r="C8" s="13" t="s">
         <v>121</v>
       </c>
-      <c r="C8" s="14" t="s">
+      <c r="D8" s="14" t="s">
         <v>122</v>
       </c>
-      <c r="D8" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E8" s="13" t="s">
+      <c r="E8" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F8" s="13" t="s">
         <v>123</v>
       </c>
-      <c r="F8" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="2:11">
-      <c r="B9" s="13" t="s">
+      <c r="G8" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="3:12">
+      <c r="C9" s="13" t="s">
         <v>121</v>
       </c>
-      <c r="C9" s="14" t="s">
+      <c r="D9" s="14" t="s">
         <v>122</v>
       </c>
-      <c r="D9" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E9" s="13" t="s">
+      <c r="E9" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F9" s="13" t="s">
         <v>123</v>
       </c>
-      <c r="F9" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="2:11">
-      <c r="B10" s="13" t="s">
+      <c r="G9" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="3:12">
+      <c r="C10" s="13" t="s">
         <v>121</v>
       </c>
-      <c r="C10" s="14" t="s">
+      <c r="D10" s="14" t="s">
         <v>122</v>
       </c>
-      <c r="D10" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E10" s="13" t="s">
+      <c r="E10" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F10" s="13" t="s">
         <v>123</v>
       </c>
-      <c r="F10" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="2:11">
-      <c r="B11" s="13" t="s">
+      <c r="G10" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="3:12">
+      <c r="C11" s="13" t="s">
         <v>121</v>
       </c>
-      <c r="C11" s="14" t="s">
+      <c r="D11" s="14" t="s">
         <v>122</v>
       </c>
-      <c r="D11" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E11" s="13" t="s">
+      <c r="E11" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F11" s="13" t="s">
         <v>123</v>
       </c>
-      <c r="F11" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="2:11">
-      <c r="B12" s="13" t="s">
+      <c r="G11" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="3:12">
+      <c r="C12" s="13" t="s">
         <v>121</v>
       </c>
-      <c r="C12" s="14" t="s">
+      <c r="D12" s="14" t="s">
         <v>122</v>
       </c>
-      <c r="D12" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E12" s="13" t="s">
+      <c r="E12" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F12" s="13" t="s">
         <v>123</v>
       </c>
-      <c r="F12" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="2:11">
-      <c r="B13" s="13" t="s">
+      <c r="G12" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="3:12">
+      <c r="C13" s="13" t="s">
         <v>121</v>
       </c>
-      <c r="C13" s="14" t="s">
+      <c r="D13" s="14" t="s">
         <v>122</v>
       </c>
-      <c r="D13" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E13" s="13" t="s">
+      <c r="E13" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F13" s="13" t="s">
         <v>123</v>
       </c>
-      <c r="F13" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="2:11">
-      <c r="B14" s="13" t="s">
+      <c r="G13" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="3:12">
+      <c r="C14" s="13" t="s">
         <v>121</v>
       </c>
-      <c r="C14" s="14" t="s">
+      <c r="D14" s="14" t="s">
         <v>122</v>
       </c>
-      <c r="D14" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E14" s="13" t="s">
+      <c r="E14" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F14" s="13" t="s">
         <v>123</v>
       </c>
-      <c r="F14" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="2:11">
-      <c r="B15" s="13" t="s">
+      <c r="G14" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="3:12">
+      <c r="C15" s="13" t="s">
         <v>121</v>
       </c>
-      <c r="C15" s="14" t="s">
+      <c r="D15" s="14" t="s">
         <v>122</v>
       </c>
-      <c r="D15" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E15" s="13" t="s">
+      <c r="E15" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F15" s="13" t="s">
         <v>123</v>
       </c>
-      <c r="F15" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="2:11">
-      <c r="B16" s="13" t="s">
+      <c r="G15" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="3:12">
+      <c r="C16" s="13" t="s">
         <v>121</v>
       </c>
-      <c r="C16" s="14" t="s">
+      <c r="D16" s="14" t="s">
         <v>122</v>
       </c>
-      <c r="D16" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E16" s="13" t="s">
+      <c r="E16" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F16" s="13" t="s">
         <v>123</v>
       </c>
-      <c r="F16" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17" spans="2:6">
-      <c r="B17" s="13" t="s">
+      <c r="G16" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="3:7">
+      <c r="C17" s="13" t="s">
         <v>121</v>
       </c>
-      <c r="C17" s="14" t="s">
+      <c r="D17" s="14" t="s">
         <v>122</v>
       </c>
-      <c r="D17" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E17" s="13" t="s">
+      <c r="E17" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F17" s="13" t="s">
         <v>123</v>
       </c>
-      <c r="F17" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18" spans="2:6">
-      <c r="B18" s="13" t="s">
+      <c r="G17" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="3:7">
+      <c r="C18" s="13" t="s">
         <v>50</v>
       </c>
-      <c r="C18" s="14" t="s">
+      <c r="D18" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="D18" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E18" s="13" t="s">
+      <c r="E18" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F18" s="13" t="s">
         <v>124</v>
       </c>
-      <c r="F18" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19" spans="2:6">
-      <c r="B19" s="13" t="s">
+      <c r="G18" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="3:7">
+      <c r="C19" s="13" t="s">
         <v>50</v>
       </c>
-      <c r="C19" s="14" t="s">
+      <c r="D19" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="D19" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E19" s="13" t="s">
+      <c r="E19" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F19" s="13" t="s">
         <v>124</v>
       </c>
-      <c r="F19" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="20" spans="2:6">
-      <c r="B20" s="13" t="s">
+      <c r="G19" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="3:7">
+      <c r="C20" s="13" t="s">
         <v>121</v>
       </c>
-      <c r="C20" s="14" t="s">
+      <c r="D20" s="14" t="s">
         <v>122</v>
       </c>
-      <c r="D20" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E20" s="13" t="s">
+      <c r="E20" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F20" s="13" t="s">
         <v>125</v>
       </c>
-      <c r="F20" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21" spans="2:6">
-      <c r="B21" s="13" t="s">
+      <c r="G20" s="15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="3:7">
+      <c r="C21" s="13" t="s">
         <v>121</v>
       </c>
-      <c r="C21" s="14" t="s">
+      <c r="D21" s="14" t="s">
         <v>122</v>
       </c>
-      <c r="D21" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E21" s="13" t="s">
+      <c r="E21" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F21" s="13" t="s">
         <v>125</v>
       </c>
-      <c r="F21" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22" spans="2:6">
-      <c r="B22" s="13" t="s">
+      <c r="G21" s="15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="3:7">
+      <c r="C22" s="13" t="s">
         <v>121</v>
       </c>
-      <c r="C22" s="14" t="s">
+      <c r="D22" s="14" t="s">
         <v>122</v>
       </c>
-      <c r="D22" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E22" s="13" t="s">
+      <c r="E22" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F22" s="13" t="s">
         <v>125</v>
       </c>
-      <c r="F22" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23" spans="2:6">
-      <c r="B23" s="13" t="s">
+      <c r="G22" s="15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="3:7">
+      <c r="C23" s="13" t="s">
         <v>121</v>
       </c>
-      <c r="C23" s="14" t="s">
+      <c r="D23" s="14" t="s">
         <v>122</v>
       </c>
-      <c r="D23" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E23" s="13" t="s">
+      <c r="E23" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F23" s="13" t="s">
         <v>125</v>
       </c>
-      <c r="F23" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="24" spans="2:6">
-      <c r="B24" s="13" t="s">
+      <c r="G23" s="15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="3:7">
+      <c r="C24" s="13" t="s">
         <v>121</v>
       </c>
-      <c r="C24" s="14" t="s">
+      <c r="D24" s="14" t="s">
         <v>122</v>
       </c>
-      <c r="D24" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E24" s="13" t="s">
+      <c r="E24" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F24" s="13" t="s">
         <v>125</v>
       </c>
-      <c r="F24" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="25" spans="2:6">
-      <c r="B25" s="13" t="s">
+      <c r="G24" s="15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="3:7">
+      <c r="C25" s="13" t="s">
         <v>126</v>
       </c>
-      <c r="C25" s="14" t="s">
+      <c r="D25" s="14" t="s">
         <v>127</v>
       </c>
-      <c r="D25" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E25" s="13" t="s">
+      <c r="E25" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F25" s="13" t="s">
         <v>128</v>
       </c>
-      <c r="F25" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="26" spans="2:6">
-      <c r="B26" s="13" t="s">
+      <c r="G25" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="3:7">
+      <c r="C26" s="13" t="s">
         <v>121</v>
       </c>
-      <c r="C26" s="14" t="s">
+      <c r="D26" s="14" t="s">
         <v>122</v>
       </c>
-      <c r="D26" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E26" s="13" t="s">
+      <c r="E26" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F26" s="13" t="s">
         <v>129</v>
       </c>
-      <c r="F26" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="27" spans="2:6">
-      <c r="B27" s="13" t="s">
+      <c r="G26" s="15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="3:7">
+      <c r="C27" s="13" t="s">
         <v>121</v>
       </c>
-      <c r="C27" s="14" t="s">
+      <c r="D27" s="14" t="s">
         <v>122</v>
       </c>
-      <c r="D27" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E27" s="13" t="s">
+      <c r="E27" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F27" s="13" t="s">
         <v>129</v>
       </c>
-      <c r="F27" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="28" spans="2:6">
-      <c r="B28" s="13" t="s">
+      <c r="G27" s="15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="3:7">
+      <c r="C28" s="13" t="s">
         <v>121</v>
       </c>
-      <c r="C28" s="14" t="s">
+      <c r="D28" s="14" t="s">
         <v>122</v>
       </c>
-      <c r="D28" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E28" s="13" t="s">
+      <c r="E28" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F28" s="13" t="s">
         <v>129</v>
       </c>
-      <c r="F28" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="29" spans="2:6">
-      <c r="B29" s="13" t="s">
+      <c r="G28" s="15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="3:7">
+      <c r="C29" s="13" t="s">
         <v>121</v>
       </c>
-      <c r="C29" s="14" t="s">
+      <c r="D29" s="14" t="s">
         <v>122</v>
       </c>
-      <c r="D29" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E29" s="13" t="s">
+      <c r="E29" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F29" s="13" t="s">
         <v>130</v>
       </c>
-      <c r="F29" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="30" spans="2:6">
-      <c r="B30" s="13" t="s">
+      <c r="G29" s="15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="3:7">
+      <c r="C30" s="13" t="s">
         <v>121</v>
       </c>
-      <c r="C30" s="14" t="s">
+      <c r="D30" s="14" t="s">
         <v>122</v>
       </c>
-      <c r="D30" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E30" s="13" t="s">
+      <c r="E30" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F30" s="13" t="s">
         <v>130</v>
       </c>
-      <c r="F30" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="31" spans="2:6">
-      <c r="B31" s="13" t="s">
+      <c r="G30" s="15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="3:7">
+      <c r="C31" s="13" t="s">
         <v>121</v>
       </c>
-      <c r="C31" s="14" t="s">
+      <c r="D31" s="14" t="s">
         <v>122</v>
       </c>
-      <c r="D31" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E31" s="13" t="s">
+      <c r="E31" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F31" s="13" t="s">
         <v>130</v>
       </c>
-      <c r="F31" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="32" spans="2:6">
-      <c r="B32" s="13" t="s">
+      <c r="G31" s="15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="3:7">
+      <c r="C32" s="13" t="s">
         <v>121</v>
       </c>
-      <c r="C32" s="14" t="s">
+      <c r="D32" s="14" t="s">
         <v>122</v>
       </c>
-      <c r="D32" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E32" s="13" t="s">
+      <c r="E32" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F32" s="13" t="s">
         <v>131</v>
       </c>
-      <c r="F32" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="33" spans="2:6">
-      <c r="B33" s="13" t="s">
+      <c r="G32" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="3:7">
+      <c r="C33" s="13" t="s">
         <v>121</v>
       </c>
-      <c r="C33" s="14" t="s">
+      <c r="D33" s="14" t="s">
         <v>122</v>
       </c>
-      <c r="D33" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E33" s="13" t="s">
+      <c r="E33" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F33" s="13" t="s">
         <v>131</v>
       </c>
-      <c r="F33" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="34" spans="2:6">
-      <c r="B34" s="13" t="s">
+      <c r="G33" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="3:7">
+      <c r="C34" s="13" t="s">
         <v>121</v>
       </c>
-      <c r="C34" s="14" t="s">
+      <c r="D34" s="14" t="s">
         <v>122</v>
       </c>
-      <c r="D34" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E34" s="13" t="s">
+      <c r="E34" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F34" s="13" t="s">
         <v>131</v>
       </c>
-      <c r="F34" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="35" spans="2:6">
-      <c r="B35" s="13" t="s">
+      <c r="G34" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="3:7">
+      <c r="C35" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="C35" s="14" t="s">
+      <c r="D35" s="14" t="s">
         <v>119</v>
       </c>
-      <c r="D35" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E35" s="13" t="s">
+      <c r="E35" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F35" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="F35" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="36" spans="2:6">
-      <c r="B36" s="13" t="s">
+      <c r="G35" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="3:7">
+      <c r="C36" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="C36" s="14" t="s">
+      <c r="D36" s="14" t="s">
         <v>119</v>
       </c>
-      <c r="D36" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E36" s="13" t="s">
+      <c r="E36" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F36" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="F36" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="37" spans="2:6">
-      <c r="B37" s="13" t="s">
+      <c r="G36" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="3:7">
+      <c r="C37" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="C37" s="14" t="s">
+      <c r="D37" s="14" t="s">
         <v>119</v>
       </c>
-      <c r="D37" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E37" s="13" t="s">
+      <c r="E37" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F37" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="F37" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="38" spans="2:6">
-      <c r="B38" s="13" t="s">
+      <c r="G37" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="3:7">
+      <c r="C38" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="C38" s="14" t="s">
+      <c r="D38" s="14" t="s">
         <v>119</v>
       </c>
-      <c r="D38" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E38" s="13" t="s">
+      <c r="E38" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F38" s="13" t="s">
         <v>133</v>
       </c>
-      <c r="F38" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="39" spans="2:6">
-      <c r="B39" s="13" t="s">
+      <c r="G38" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" spans="3:7">
+      <c r="C39" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="C39" s="14" t="s">
+      <c r="D39" s="14" t="s">
         <v>119</v>
       </c>
-      <c r="D39" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E39" s="13" t="s">
+      <c r="E39" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F39" s="13" t="s">
         <v>133</v>
       </c>
-      <c r="F39" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="40" spans="2:6">
-      <c r="B40" s="13" t="s">
+      <c r="G39" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40" spans="3:7">
+      <c r="C40" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="C40" s="14" t="s">
+      <c r="D40" s="14" t="s">
         <v>119</v>
       </c>
-      <c r="D40" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E40" s="13" t="s">
+      <c r="E40" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F40" s="13" t="s">
         <v>133</v>
       </c>
-      <c r="F40" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="41" spans="2:6">
-      <c r="B41" s="13" t="s">
+      <c r="G40" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" spans="3:7">
+      <c r="C41" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="C41" s="14" t="s">
+      <c r="D41" s="14" t="s">
         <v>119</v>
       </c>
-      <c r="D41" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E41" s="13" t="s">
+      <c r="E41" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F41" s="13" t="s">
         <v>133</v>
       </c>
-      <c r="F41" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="42" spans="2:6">
-      <c r="B42" s="13" t="s">
+      <c r="G41" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42" spans="3:7">
+      <c r="C42" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="C42" s="14" t="s">
+      <c r="D42" s="14" t="s">
         <v>119</v>
       </c>
-      <c r="D42" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E42" s="13" t="s">
+      <c r="E42" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F42" s="13" t="s">
         <v>133</v>
       </c>
-      <c r="F42" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="43" spans="2:6">
-      <c r="B43" s="13" t="s">
+      <c r="G42" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43" spans="3:7">
+      <c r="C43" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="C43" s="14" t="s">
+      <c r="D43" s="14" t="s">
         <v>119</v>
       </c>
-      <c r="D43" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E43" s="13" t="s">
+      <c r="E43" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F43" s="13" t="s">
         <v>133</v>
       </c>
-      <c r="F43" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="44" spans="2:6">
-      <c r="B44" s="13" t="s">
+      <c r="G43" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44" spans="3:7">
+      <c r="C44" s="13" t="s">
         <v>50</v>
       </c>
-      <c r="C44" s="14" t="s">
+      <c r="D44" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="D44" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E44" s="13" t="s">
+      <c r="E44" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F44" s="13" t="s">
         <v>134</v>
       </c>
-      <c r="F44" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="45" spans="2:6">
-      <c r="B45" s="13" t="s">
+      <c r="G44" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45" spans="3:7">
+      <c r="C45" s="13" t="s">
         <v>50</v>
       </c>
-      <c r="C45" s="14" t="s">
+      <c r="D45" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="D45" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E45" s="13" t="s">
+      <c r="E45" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F45" s="13" t="s">
         <v>134</v>
       </c>
-      <c r="F45" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="46" spans="2:6">
-      <c r="B46" s="13" t="s">
+      <c r="G45" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46" spans="3:7">
+      <c r="C46" s="13" t="s">
         <v>50</v>
       </c>
-      <c r="C46" s="14" t="s">
+      <c r="D46" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="D46" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E46" s="13" t="s">
+      <c r="E46" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F46" s="13" t="s">
         <v>134</v>
       </c>
-      <c r="F46" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="47" spans="2:6">
-      <c r="B47" s="13" t="s">
+      <c r="G46" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47" spans="3:7">
+      <c r="C47" s="13" t="s">
         <v>50</v>
       </c>
-      <c r="C47" s="14" t="s">
+      <c r="D47" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="D47" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E47" s="13" t="s">
+      <c r="E47" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F47" s="13" t="s">
         <v>134</v>
       </c>
-      <c r="F47" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="48" spans="2:6">
-      <c r="B48" s="13" t="s">
+      <c r="G47" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48" spans="3:7">
+      <c r="C48" s="13" t="s">
         <v>50</v>
       </c>
-      <c r="C48" s="14" t="s">
+      <c r="D48" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="D48" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E48" s="13" t="s">
+      <c r="E48" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F48" s="13" t="s">
         <v>134</v>
       </c>
-      <c r="F48" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="49" spans="2:6">
-      <c r="B49" s="13" t="s">
+      <c r="G48" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49" spans="3:7">
+      <c r="C49" s="13" t="s">
         <v>50</v>
       </c>
-      <c r="C49" s="14" t="s">
+      <c r="D49" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="D49" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E49" s="13" t="s">
+      <c r="E49" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F49" s="13" t="s">
         <v>134</v>
       </c>
-      <c r="F49" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="50" spans="2:6">
-      <c r="B50" s="13" t="s">
+      <c r="G49" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50" spans="3:7">
+      <c r="C50" s="13" t="s">
         <v>50</v>
       </c>
-      <c r="C50" s="14" t="s">
+      <c r="D50" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="D50" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E50" s="13" t="s">
+      <c r="E50" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F50" s="13" t="s">
         <v>135</v>
       </c>
-      <c r="F50" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="51" spans="2:6">
-      <c r="B51" s="13" t="s">
+      <c r="G50" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51" spans="3:7">
+      <c r="C51" s="13" t="s">
         <v>50</v>
       </c>
-      <c r="C51" s="14" t="s">
+      <c r="D51" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="D51" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E51" s="13" t="s">
+      <c r="E51" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F51" s="13" t="s">
         <v>135</v>
       </c>
-      <c r="F51" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="52" spans="2:6">
-      <c r="B52" s="13" t="s">
+      <c r="G51" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52" spans="3:7">
+      <c r="C52" s="13" t="s">
         <v>121</v>
       </c>
-      <c r="C52" s="14" t="s">
+      <c r="D52" s="14" t="s">
         <v>122</v>
       </c>
-      <c r="D52" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E52" s="13" t="s">
+      <c r="E52" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F52" s="13" t="s">
         <v>136</v>
       </c>
-      <c r="F52" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="53" spans="2:6">
-      <c r="B53" s="13" t="s">
+      <c r="G52" s="15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53" spans="3:7">
+      <c r="C53" s="13" t="s">
         <v>121</v>
       </c>
-      <c r="C53" s="14" t="s">
+      <c r="D53" s="14" t="s">
         <v>122</v>
       </c>
-      <c r="D53" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E53" s="13" t="s">
+      <c r="E53" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F53" s="13" t="s">
         <v>136</v>
       </c>
-      <c r="F53" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="54" spans="2:6">
-      <c r="B54" s="13" t="s">
+      <c r="G53" s="15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54" spans="3:7">
+      <c r="C54" s="13" t="s">
         <v>121</v>
       </c>
-      <c r="C54" s="14" t="s">
+      <c r="D54" s="14" t="s">
         <v>122</v>
       </c>
-      <c r="D54" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E54" s="13" t="s">
+      <c r="E54" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F54" s="13" t="s">
         <v>136</v>
       </c>
-      <c r="F54" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="55" spans="2:6">
-      <c r="B55" s="13"/>
-      <c r="C55" s="14"/>
-      <c r="D55" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E55" s="13" t="s">
+      <c r="G54" s="15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55" spans="3:7">
+      <c r="C55" s="13"/>
+      <c r="D55" s="14"/>
+      <c r="E55" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F55" s="13" t="s">
         <v>137</v>
       </c>
-      <c r="F55" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="56" spans="2:6">
-      <c r="B56" s="13" t="s">
+      <c r="G55" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56" spans="3:7">
+      <c r="C56" s="13" t="s">
         <v>121</v>
       </c>
-      <c r="C56" s="14" t="s">
+      <c r="D56" s="14" t="s">
         <v>138</v>
       </c>
-      <c r="D56" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E56" s="13" t="s">
+      <c r="E56" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F56" s="13" t="s">
         <v>139</v>
       </c>
-      <c r="F56" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="57" spans="2:6">
-      <c r="B57" s="13" t="s">
+      <c r="G56" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57" spans="3:7">
+      <c r="C57" s="13" t="s">
         <v>121</v>
       </c>
-      <c r="C57" s="14" t="s">
+      <c r="D57" s="14" t="s">
         <v>138</v>
       </c>
-      <c r="D57" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E57" s="13" t="s">
+      <c r="E57" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F57" s="13" t="s">
         <v>139</v>
       </c>
-      <c r="F57" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="58" spans="2:6">
-      <c r="B58" s="13" t="s">
+      <c r="G57" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="58" spans="3:7">
+      <c r="C58" s="13" t="s">
         <v>121</v>
       </c>
-      <c r="C58" s="14" t="s">
+      <c r="D58" s="14" t="s">
         <v>138</v>
       </c>
-      <c r="D58" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E58" s="13" t="s">
+      <c r="E58" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F58" s="13" t="s">
         <v>139</v>
       </c>
-      <c r="F58" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="59" spans="2:6">
-      <c r="B59" s="13" t="s">
+      <c r="G58" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="59" spans="3:7">
+      <c r="C59" s="13" t="s">
         <v>50</v>
       </c>
-      <c r="C59" s="14" t="s">
+      <c r="D59" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="D59" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E59" s="13" t="s">
+      <c r="E59" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F59" s="13" t="s">
         <v>140</v>
       </c>
-      <c r="F59" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="60" spans="2:6">
-      <c r="B60" s="13" t="s">
+      <c r="G59" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="60" spans="3:7">
+      <c r="C60" s="13" t="s">
         <v>50</v>
       </c>
-      <c r="C60" s="14" t="s">
+      <c r="D60" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="D60" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E60" s="13" t="s">
+      <c r="E60" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F60" s="13" t="s">
         <v>140</v>
       </c>
-      <c r="F60" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="61" spans="2:6">
-      <c r="B61" s="13" t="s">
+      <c r="G60" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="61" spans="3:7">
+      <c r="C61" s="13" t="s">
         <v>50</v>
       </c>
-      <c r="C61" s="14" t="s">
+      <c r="D61" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="D61" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E61" s="13" t="s">
+      <c r="E61" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F61" s="13" t="s">
         <v>140</v>
       </c>
-      <c r="F61" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="62" spans="2:6">
-      <c r="B62" s="13" t="s">
+      <c r="G61" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="62" spans="3:7">
+      <c r="C62" s="13" t="s">
         <v>50</v>
       </c>
-      <c r="C62" s="14" t="s">
+      <c r="D62" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="D62" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E62" s="13" t="s">
+      <c r="E62" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F62" s="13" t="s">
         <v>140</v>
       </c>
-      <c r="F62" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="63" spans="2:6">
-      <c r="B63" s="13" t="s">
+      <c r="G62" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="63" spans="3:7">
+      <c r="C63" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="C63" s="14" t="s">
+      <c r="D63" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="D63" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E63" s="13" t="s">
+      <c r="E63" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F63" s="13" t="s">
         <v>140</v>
       </c>
-      <c r="F63" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="64" spans="2:6">
-      <c r="B64" s="13" t="s">
+      <c r="G63" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="64" spans="3:7">
+      <c r="C64" s="13" t="s">
         <v>50</v>
       </c>
-      <c r="C64" s="14" t="s">
+      <c r="D64" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="D64" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E64" s="13" t="s">
+      <c r="E64" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F64" s="13" t="s">
         <v>140</v>
       </c>
-      <c r="F64" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="65" spans="2:6">
-      <c r="B65" s="13" t="s">
+      <c r="G64" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="65" spans="3:7">
+      <c r="C65" s="13" t="s">
         <v>50</v>
       </c>
-      <c r="C65" s="14" t="s">
+      <c r="D65" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="D65" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E65" s="13" t="s">
+      <c r="E65" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F65" s="13" t="s">
         <v>140</v>
       </c>
-      <c r="F65" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="66" spans="2:6">
-      <c r="B66" s="13" t="s">
+      <c r="G65" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="66" spans="3:7">
+      <c r="C66" s="13" t="s">
         <v>50</v>
       </c>
-      <c r="C66" s="14" t="s">
+      <c r="D66" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="D66" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E66" s="13" t="s">
+      <c r="E66" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F66" s="13" t="s">
         <v>140</v>
       </c>
-      <c r="F66" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="67" spans="2:6">
-      <c r="B67" s="13" t="s">
+      <c r="G66" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="67" spans="3:7">
+      <c r="C67" s="13" t="s">
         <v>50</v>
       </c>
-      <c r="C67" s="14" t="s">
+      <c r="D67" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="D67" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E67" s="13" t="s">
+      <c r="E67" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F67" s="13" t="s">
         <v>140</v>
       </c>
-      <c r="F67" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="68" spans="2:6">
-      <c r="B68" s="13" t="s">
+      <c r="G67" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="68" spans="3:7">
+      <c r="C68" s="13" t="s">
         <v>121</v>
       </c>
-      <c r="C68" s="14" t="s">
+      <c r="D68" s="14" t="s">
         <v>122</v>
       </c>
-      <c r="D68" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E68" s="13" t="s">
+      <c r="E68" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F68" s="13" t="s">
         <v>141</v>
       </c>
-      <c r="F68" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="69" spans="2:6">
-      <c r="B69" s="13" t="s">
+      <c r="G68" s="15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="69" spans="3:7">
+      <c r="C69" s="13" t="s">
         <v>121</v>
       </c>
-      <c r="C69" s="14" t="s">
+      <c r="D69" s="14" t="s">
         <v>122</v>
       </c>
-      <c r="D69" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E69" s="13" t="s">
+      <c r="E69" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F69" s="13" t="s">
         <v>141</v>
       </c>
-      <c r="F69" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="70" spans="2:6">
-      <c r="B70" s="13" t="s">
+      <c r="G69" s="15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="70" spans="3:7">
+      <c r="C70" s="13" t="s">
         <v>121</v>
       </c>
-      <c r="C70" s="14" t="s">
+      <c r="D70" s="14" t="s">
         <v>122</v>
       </c>
-      <c r="D70" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E70" s="13" t="s">
+      <c r="E70" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F70" s="13" t="s">
         <v>141</v>
       </c>
-      <c r="F70" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="71" spans="2:6">
-      <c r="B71" s="13" t="s">
+      <c r="G70" s="15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="71" spans="3:7">
+      <c r="C71" s="13" t="s">
         <v>121</v>
       </c>
-      <c r="C71" s="14" t="s">
+      <c r="D71" s="14" t="s">
         <v>122</v>
       </c>
-      <c r="D71" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E71" s="13" t="s">
+      <c r="E71" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F71" s="13" t="s">
         <v>141</v>
       </c>
-      <c r="F71" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="72" spans="2:6">
-      <c r="B72" s="13" t="s">
+      <c r="G71" s="15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="72" spans="3:7">
+      <c r="C72" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="C72" s="14" t="s">
+      <c r="D72" s="14" t="s">
         <v>119</v>
       </c>
-      <c r="D72" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E72" s="13" t="s">
+      <c r="E72" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F72" s="13" t="s">
         <v>142</v>
       </c>
-      <c r="F72" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="73" spans="2:6">
-      <c r="B73" s="13" t="s">
+      <c r="G72" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="73" spans="3:7">
+      <c r="C73" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="C73" s="14" t="s">
+      <c r="D73" s="14" t="s">
         <v>119</v>
       </c>
-      <c r="D73" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E73" s="13" t="s">
+      <c r="E73" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F73" s="13" t="s">
         <v>142</v>
       </c>
-      <c r="F73" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="74" spans="2:6">
-      <c r="B74" s="13" t="s">
+      <c r="G73" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="74" spans="3:7">
+      <c r="C74" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="C74" s="14" t="s">
+      <c r="D74" s="14" t="s">
         <v>119</v>
       </c>
-      <c r="D74" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E74" s="13" t="s">
+      <c r="E74" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F74" s="13" t="s">
         <v>142</v>
       </c>
-      <c r="F74" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="75" spans="2:6">
-      <c r="B75" s="13" t="s">
+      <c r="G74" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="75" spans="3:7">
+      <c r="C75" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="C75" s="14" t="s">
+      <c r="D75" s="14" t="s">
         <v>119</v>
       </c>
-      <c r="D75" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E75" s="13" t="s">
+      <c r="E75" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F75" s="13" t="s">
         <v>142</v>
       </c>
-      <c r="F75" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="76" spans="2:6">
-      <c r="B76" s="13" t="s">
+      <c r="G75" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="76" spans="3:7">
+      <c r="C76" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="C76" s="14" t="s">
+      <c r="D76" s="14" t="s">
         <v>119</v>
       </c>
-      <c r="D76" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E76" s="13" t="s">
+      <c r="E76" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F76" s="13" t="s">
         <v>142</v>
       </c>
-      <c r="F76" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="77" spans="2:6">
-      <c r="B77" s="13" t="s">
+      <c r="G76" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="77" spans="3:7">
+      <c r="C77" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="C77" s="14" t="s">
+      <c r="D77" s="14" t="s">
         <v>119</v>
       </c>
-      <c r="D77" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E77" s="13" t="s">
+      <c r="E77" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F77" s="13" t="s">
         <v>142</v>
       </c>
-      <c r="F77" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="78" spans="2:6">
-      <c r="B78" s="13" t="s">
+      <c r="G77" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="78" spans="3:7">
+      <c r="C78" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="C78" s="14" t="s">
+      <c r="D78" s="14" t="s">
         <v>119</v>
       </c>
-      <c r="D78" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E78" s="13" t="s">
+      <c r="E78" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F78" s="13" t="s">
         <v>142</v>
       </c>
-      <c r="F78" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="79" spans="2:6">
-      <c r="B79" s="13" t="s">
+      <c r="G78" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="79" spans="3:7">
+      <c r="C79" s="13" t="s">
         <v>121</v>
       </c>
-      <c r="C79" s="14" t="s">
+      <c r="D79" s="14" t="s">
         <v>138</v>
       </c>
-      <c r="D79" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E79" s="13" t="s">
+      <c r="E79" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F79" s="13" t="s">
         <v>143</v>
       </c>
-      <c r="F79" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="80" spans="2:6">
-      <c r="B80" s="13" t="s">
+      <c r="G79" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="80" spans="3:7">
+      <c r="C80" s="13" t="s">
         <v>121</v>
       </c>
-      <c r="C80" s="14" t="s">
+      <c r="D80" s="14" t="s">
         <v>138</v>
       </c>
-      <c r="D80" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E80" s="13" t="s">
+      <c r="E80" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F80" s="13" t="s">
         <v>143</v>
       </c>
-      <c r="F80" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="81" spans="2:6">
-      <c r="B81" s="13" t="s">
+      <c r="G80" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="81" spans="3:7">
+      <c r="C81" s="13" t="s">
         <v>121</v>
       </c>
-      <c r="C81" s="14" t="s">
+      <c r="D81" s="14" t="s">
         <v>138</v>
       </c>
-      <c r="D81" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E81" s="13" t="s">
+      <c r="E81" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F81" s="13" t="s">
         <v>143</v>
       </c>
-      <c r="F81" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="82" spans="2:6">
-      <c r="B82" s="13" t="s">
+      <c r="G81" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="82" spans="3:7">
+      <c r="C82" s="13" t="s">
         <v>121</v>
       </c>
-      <c r="C82" s="14" t="s">
+      <c r="D82" s="14" t="s">
         <v>122</v>
       </c>
-      <c r="D82" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E82" s="13" t="s">
+      <c r="E82" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F82" s="13" t="s">
         <v>144</v>
       </c>
-      <c r="F82" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="83" spans="2:6">
-      <c r="B83" s="13" t="s">
+      <c r="G82" s="15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="83" spans="3:7">
+      <c r="C83" s="13" t="s">
         <v>126</v>
       </c>
-      <c r="C83" s="14" t="s">
+      <c r="D83" s="14" t="s">
         <v>127</v>
       </c>
-      <c r="D83" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E83" s="13" t="s">
+      <c r="E83" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F83" s="13" t="s">
         <v>145</v>
       </c>
-      <c r="F83" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="84" spans="2:6">
-      <c r="B84" s="13" t="s">
+      <c r="G83" s="15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="84" spans="3:7">
+      <c r="C84" s="13" t="s">
         <v>126</v>
       </c>
-      <c r="C84" s="14" t="s">
+      <c r="D84" s="14" t="s">
         <v>127</v>
       </c>
-      <c r="D84" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E84" s="13" t="s">
+      <c r="E84" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F84" s="13" t="s">
         <v>146</v>
       </c>
-      <c r="F84" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="85" spans="2:6">
-      <c r="B85" s="13" t="s">
+      <c r="G84" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="85" spans="3:7">
+      <c r="C85" s="13" t="s">
         <v>121</v>
       </c>
-      <c r="C85" s="14" t="s">
+      <c r="D85" s="14" t="s">
         <v>138</v>
       </c>
-      <c r="D85" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E85" s="13" t="s">
+      <c r="E85" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F85" s="13" t="s">
         <v>147</v>
       </c>
-      <c r="F85" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="86" spans="2:6">
-      <c r="B86" s="13" t="s">
+      <c r="G85" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="86" spans="3:7">
+      <c r="C86" s="13" t="s">
         <v>121</v>
       </c>
-      <c r="C86" s="14" t="s">
+      <c r="D86" s="14" t="s">
         <v>138</v>
       </c>
-      <c r="D86" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E86" s="13" t="s">
+      <c r="E86" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F86" s="13" t="s">
         <v>147</v>
       </c>
-      <c r="F86" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="87" spans="2:6">
-      <c r="B87" s="13"/>
-      <c r="C87" s="14"/>
-      <c r="D87" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E87" s="13" t="s">
+      <c r="G86" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="87" spans="3:7">
+      <c r="C87" s="13"/>
+      <c r="D87" s="14"/>
+      <c r="E87" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F87" s="13" t="s">
         <v>148</v>
       </c>
-      <c r="F87" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="88" spans="2:6">
-      <c r="B88" s="13" t="s">
+      <c r="G87" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="88" spans="3:7">
+      <c r="C88" s="13" t="s">
         <v>126</v>
       </c>
-      <c r="C88" s="14" t="s">
+      <c r="D88" s="14" t="s">
         <v>127</v>
       </c>
-      <c r="D88" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E88" s="13" t="s">
+      <c r="E88" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F88" s="13" t="s">
         <v>149</v>
       </c>
-      <c r="F88" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="89" spans="2:6">
-      <c r="B89" s="13" t="s">
+      <c r="G88" s="15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="89" spans="3:7">
+      <c r="C89" s="13" t="s">
         <v>121</v>
       </c>
-      <c r="C89" s="14" t="s">
+      <c r="D89" s="14" t="s">
         <v>138</v>
       </c>
-      <c r="D89" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E89" s="13" t="s">
+      <c r="E89" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F89" s="13" t="s">
         <v>150</v>
       </c>
-      <c r="F89" s="15">
+      <c r="G89" s="15">
         <v>1</v>
       </c>
     </row>
@@ -4595,7 +4595,7 @@
       <c r="M9" s="13" t="s">
         <v>161</v>
       </c>
-      <c r="N9" s="14">
+      <c r="N9" s="15">
         <v>1</v>
       </c>
     </row>
@@ -4883,7 +4883,7 @@
       <c r="M18" s="13" t="s">
         <v>175</v>
       </c>
-      <c r="N18" s="14">
+      <c r="N18" s="15">
         <v>1</v>
       </c>
     </row>
@@ -5003,7 +5003,7 @@
       <c r="M22" s="13" t="s">
         <v>185</v>
       </c>
-      <c r="N22" s="14">
+      <c r="N22" s="15">
         <v>1</v>
       </c>
     </row>
@@ -5223,7 +5223,7 @@
       <c r="M30" s="13" t="s">
         <v>201</v>
       </c>
-      <c r="N30" s="14">
+      <c r="N30" s="15">
         <v>1</v>
       </c>
     </row>
@@ -5505,7 +5505,7 @@
       <c r="M43" s="13" t="s">
         <v>215</v>
       </c>
-      <c r="N43" s="14">
+      <c r="N43" s="15">
         <v>1</v>
       </c>
     </row>
@@ -5581,7 +5581,7 @@
       <c r="M47" s="13" t="s">
         <v>219</v>
       </c>
-      <c r="N47" s="14">
+      <c r="N47" s="15">
         <v>1</v>
       </c>
     </row>

</xml_diff>